<commit_message>
change saving receipt (headers) document
</commit_message>
<xml_diff>
--- a/PromVesClient/Templates/CardTemplate.xlsx
+++ b/PromVesClient/Templates/CardTemplate.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Клиент\PromVesClient\PromVesClient\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Клиент\PromVesClientCovdor\PromVesClient\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E892DDC-73A8-43E5-8867-763974A9883D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C28D19F-1994-4F1F-9282-80B8884FCB10}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,66 +25,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
-  <si>
-    <t>Номер вагона</t>
-  </si>
-  <si>
-    <t>Тара, т.</t>
-  </si>
-  <si>
-    <t>Нетто, т.</t>
-  </si>
-  <si>
-    <t>Брутто, т.</t>
-  </si>
-  <si>
-    <t>Разница бортов, т.</t>
-  </si>
-  <si>
-    <t>Тележка 1, т.</t>
-  </si>
-  <si>
-    <t>Тележка 2, т.</t>
-  </si>
-  <si>
-    <t>Разница тележек, т.</t>
-  </si>
-  <si>
-    <t>Левый борт, т.</t>
-  </si>
-  <si>
-    <t>Правый борт, т.</t>
-  </si>
-  <si>
-    <t>Недогруз перегруз, т.</t>
-  </si>
-  <si>
-    <t>АО «Уральский завод металлоконструкций»</t>
-  </si>
-  <si>
-    <t>Грузоподъёмность, т.</t>
-  </si>
-</sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -104,34 +55,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -140,15 +69,13 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -447,63 +374,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
+      <c r="A1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
     </row>
-    <row r="2" spans="1:12" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>4</v>
-      </c>
+    <row r="2" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
changing the creation of headings in a document
</commit_message>
<xml_diff>
--- a/PromVesClient/Templates/CardTemplate.xlsx
+++ b/PromVesClient/Templates/CardTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Клиент\PromVesClientCovdor\PromVesClient\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C28D19F-1994-4F1F-9282-80B8884FCB10}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C9FC024-5E75-4227-8B56-F8C0D843F070}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,10 +22,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -67,11 +63,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -356,7 +349,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="L1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" customWidth="1"/>
@@ -373,33 +366,11 @@
     <col min="12" max="12" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+    <row r="1" spans="12:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
+    <row r="2" spans="12:12" x14ac:dyDescent="0.25">
+      <c r="L2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>